<commit_message>
W2: final v5 on Baari, R3 closed at 8 of 10, Q10 written
B2 balance-alone rule and the D-line honesty rule added to v5, pushed to
Baari 20:38. E04 still fails (GPT-5.4 batches balance, shipment, debit),
E05 misses the M6 citation. CHANGELOG, STATUS, run log sheet updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evals/out/baari_run_log.xlsx
+++ b/evals/out/baari_run_log.xlsx
@@ -743,14 +743,14 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T14:49:30.232Z</t>
+          <t>2026-10-04T15:08:08.796Z</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>9 of 10</t>
+          <t>8 of 10</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M75"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5690,6 +5690,536 @@
       <c r="M75" s="2" t="inlineStr">
         <is>
           <t>evals/runs/R3/E04/2026-10-04T14-49-30-232Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T14:52:41.520Z</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">run_error: TimeoutError: The operation was aborted due to timeout
+    at node:internal/deps/undici/undici:15141:13
+    at process.processTicksAndRejections (node:internal/process/task_queues:103:5)
+  </t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E04/2026-10-04T14-52-41-520Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T14:54:16.870Z</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>2df30651-7732-4016-adc9-eebe18354d50</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>77809</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E02/2026-10-04T14-54-16-870Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T14:54:56.227Z</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">run_error: TimeoutError: The operation was aborted due to timeout
+    at node:internal/deps/undici/undici:15141:13
+    at process.processTicksAndRejections (node:internal/process/task_queues:103:5)
+  </t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E05/2026-10-04T14-54-56-227Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T14:57:29.025Z</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>2c4c3961-3bbd-4625-8aa8-9a01ed4460ac</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>expect:no_debit_over: debit of 10626</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>68427</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E04/2026-10-04T14-57-29-025Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T14:59:45.126Z</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>9f28c0f8-2dce-4cfb-9f4d-32d63c4d4cf1</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>expect:rule_cited: rules not cited: M6 (cited: V1 V4 V5 V5 B1 B2 M4 B4 E1 M7 B4)</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>112943</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E05/2026-10-04T14-59-45-126Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:04:23.887Z</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>5243a5f3-fc0a-4237-8842-45a9c7a87bd6</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>expect:no_debit_over: debit of 10626</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>74532</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E04/2026-10-04T15-04-23-887Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:06:02.013Z</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>5b99016f-6b9f-4a6a-905c-0b08aa2b495d</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>decisions_match_log: side effects with no decision: create_shipment, send_message</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>76163</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E04/2026-10-04T15-06-02-013Z_platform.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>azure_openai/deployment:gpt-5.4</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>v5</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>simulated</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T15:08:08.796Z</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>a3fc6ade-b589-4f9f-844d-233610e20e0c</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>expect:rule_cited: rules not cited: M6 (cited: V1 V1 V4 V5 V5 M2 B1 B2 M4 B3 E1 M7)</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>111143</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>evals/runs/R3/E05/2026-10-04T15-08-08-796Z_platform.json</t>
         </is>
       </c>
     </row>

</xml_diff>